<commit_message>
whole lotta dumb stuff
</commit_message>
<xml_diff>
--- a/Database/reports/OS Byggingar_July.xlsx
+++ b/Database/reports/OS Byggingar_July.xlsx
@@ -450,18 +450,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="2" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>3rd of July</t>
+          <t>1st of July</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -474,221 +479,1196 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Employee ID</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Task</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Task</t>
+          <t>Clock In</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Clock In</t>
+          <t>Clock Out</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Clock Out</t>
+          <t>Lunch (min)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Hours Worked</t>
+          <t>Paid Hours</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>olafur</t>
+          <t>Ólafur Sær</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Total: 8.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2nd of July</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Ólafur Sær</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Reykjavíkuvegur 60, 220 Hafnafjörður</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Total: 9.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>3rd of July</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Total: 6.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>5th of July</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Total: 4.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>6th of July</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>útivinna</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Total: 10.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>7th of July</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>útivinna</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Total: 10.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>8th of July</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>útivinna</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Total: 10.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>9th of July</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>útivinna</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Total: 8.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>10th of July</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>útivinna</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>Total: 10.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>11th of July</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Total: 4.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>17th of July</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Clock In</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Clock Out</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Lunch (min)</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Paid Hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Ólafur Sær</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Aðstöðusköpun, rekstur og stjórnun</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>11:07</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>11:07</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>olafur</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Ólafur Sær</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Reykjavíkuvegur 60, 220 Hafnafjörður</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Dalshverfi III, 230 Reykjanes</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr"/>
+      <c r="B65" s="2" t="inlineStr"/>
+      <c r="C65" s="2" t="inlineStr"/>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>Total: -0.14 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Overall Paid Hours: 78.86 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="G68" s="5" t="n"/>
+    </row>
+    <row r="69"/>
+    <row r="70">
+      <c r="A70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Task Name</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Total Hours</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Completed?</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>Aðstöðusköpun, rekstur og stjórnun</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>11:21</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>11:21</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>olafur</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Ólafur Sær</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Reykjavíkuvegur 60, 220 Hafnafjörður</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Aðstöðusköpun, rekstur og stjórnun</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>11:12</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>47.7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Total: 47.7 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Overall Total Hours: 47.7 hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="G9" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Task Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Task Name</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Total Hours</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Completed?</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Aðstöðusköpun, rekstur og stjórnun</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B72" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="C72" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Tölvuvinna/Appþróun</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>30.92</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>útivinna</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>48</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="12">
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A61:H61"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>